<commit_message>
Update substitutions September 10
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="842" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="156">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -352,30 +352,42 @@
     <t>32</t>
   </si>
   <si>
+    <t>2WA</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Wójcik Kamil</t>
+  </si>
+  <si>
     <t>26</t>
   </si>
   <si>
+    <t>1FA</t>
+  </si>
+  <si>
+    <t>Filipek Anna</t>
+  </si>
+  <si>
     <t>1TFB</t>
   </si>
   <si>
     <t>Danielewski Paweł</t>
   </si>
   <si>
+    <t>Chemia</t>
+  </si>
+  <si>
     <t>11.09.2026</t>
   </si>
   <si>
     <t>3</t>
   </si>
   <si>
-    <t>28</t>
-  </si>
-  <si>
     <t>Małecka Barbara</t>
   </si>
   <si>
-    <t>Chemia</t>
-  </si>
-  <si>
     <t>Hudziec Agnieszka</t>
   </si>
   <si>
@@ -385,9 +397,6 @@
     <t>Sałdyka Karolina</t>
   </si>
   <si>
-    <t>1FA</t>
-  </si>
-  <si>
     <t>43</t>
   </si>
   <si>
@@ -422,9 +431,6 @@
   </si>
   <si>
     <t>14:00-14:05</t>
-  </si>
-  <si>
-    <t>Wójcik Kamil</t>
   </si>
   <si>
     <t>14:50-14:55</t>
@@ -931,7 +937,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5edf3915-bad0-491f-977a-c498ca5b309e}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f5905cba-1004-41ce-85e8-c077faefae63}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -952,8 +958,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{97035fd9-5966-4286-9b08-b4899efa4cbd}">
-  <dimension ref="A1:I82"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{a4da12a8-2b8c-4c9b-96fe-b6984f3133b1}">
+  <dimension ref="A1:I87"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
@@ -2512,19 +2518,19 @@
         <v>31</v>
       </c>
       <c r="C54" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>25</v>
+        <v>110</v>
       </c>
       <c r="E54" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F54" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="G54" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="H54" t="s">
         <v>18</v>
@@ -2541,19 +2547,19 @@
         <v>31</v>
       </c>
       <c r="C55" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D55" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="E55" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="F55" t="s">
-        <v>110</v>
+        <v>97</v>
       </c>
       <c r="G55" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H55" t="s">
         <v>18</v>
@@ -2567,28 +2573,28 @@
         <v>95</v>
       </c>
       <c r="B56" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C56" t="s">
-        <v>32</v>
+        <v>13</v>
       </c>
       <c r="D56" t="s">
-        <v>33</v>
+        <v>14</v>
       </c>
       <c r="E56" t="s">
-        <v>83</v>
+        <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>92</v>
+        <v>113</v>
       </c>
       <c r="G56" t="s">
-        <v>49</v>
+        <v>100</v>
       </c>
       <c r="H56" t="s">
         <v>18</v>
       </c>
       <c r="I56" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="57" spans="1:9" ht="15">
@@ -2599,19 +2605,19 @@
         <v>44</v>
       </c>
       <c r="C57" t="s">
-        <v>24</v>
+        <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>25</v>
+        <v>114</v>
       </c>
       <c r="E57" t="s">
-        <v>47</v>
+        <v>82</v>
       </c>
       <c r="F57" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="G57" t="s">
-        <v>98</v>
+        <v>115</v>
       </c>
       <c r="H57" t="s">
         <v>18</v>
@@ -2628,25 +2634,25 @@
         <v>44</v>
       </c>
       <c r="C58" t="s">
-        <v>13</v>
+        <v>32</v>
       </c>
       <c r="D58" t="s">
-        <v>14</v>
+        <v>33</v>
       </c>
       <c r="E58" t="s">
-        <v>30</v>
+        <v>83</v>
       </c>
       <c r="F58" t="s">
-        <v>68</v>
+        <v>92</v>
       </c>
       <c r="G58" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="H58" t="s">
         <v>18</v>
       </c>
       <c r="I58" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="59" spans="1:9" ht="15">
@@ -2654,22 +2660,22 @@
         <v>95</v>
       </c>
       <c r="B59" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="C59" t="s">
-        <v>55</v>
+        <v>24</v>
       </c>
       <c r="D59" t="s">
-        <v>56</v>
+        <v>25</v>
       </c>
       <c r="E59" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="F59" t="s">
-        <v>58</v>
+        <v>97</v>
       </c>
       <c r="G59" t="s">
-        <v>64</v>
+        <v>98</v>
       </c>
       <c r="H59" t="s">
         <v>18</v>
@@ -2683,22 +2689,22 @@
         <v>95</v>
       </c>
       <c r="B60" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C60" t="s">
-        <v>55</v>
+        <v>13</v>
       </c>
       <c r="D60" t="s">
-        <v>56</v>
+        <v>14</v>
       </c>
       <c r="E60" t="s">
-        <v>63</v>
+        <v>30</v>
       </c>
       <c r="F60" t="s">
-        <v>58</v>
+        <v>68</v>
       </c>
       <c r="G60" t="s">
-        <v>64</v>
+        <v>100</v>
       </c>
       <c r="H60" t="s">
         <v>18</v>
@@ -2712,22 +2718,22 @@
         <v>95</v>
       </c>
       <c r="B61" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C61" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="D61" t="s">
-        <v>111</v>
+        <v>56</v>
       </c>
       <c r="E61" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="F61" t="s">
-        <v>97</v>
+        <v>58</v>
       </c>
       <c r="G61" t="s">
-        <v>112</v>
+        <v>64</v>
       </c>
       <c r="H61" t="s">
         <v>18</v>
@@ -2741,22 +2747,22 @@
         <v>95</v>
       </c>
       <c r="B62" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
       <c r="C62" t="s">
-        <v>55</v>
+        <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>62</v>
+        <v>116</v>
       </c>
       <c r="E62" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="F62" t="s">
-        <v>58</v>
+        <v>111</v>
       </c>
       <c r="G62" t="s">
-        <v>64</v>
+        <v>117</v>
       </c>
       <c r="H62" t="s">
         <v>18</v>
@@ -2770,22 +2776,22 @@
         <v>95</v>
       </c>
       <c r="B63" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C63" t="s">
-        <v>24</v>
+        <v>55</v>
       </c>
       <c r="D63" t="s">
-        <v>91</v>
+        <v>56</v>
       </c>
       <c r="E63" t="s">
-        <v>26</v>
+        <v>63</v>
       </c>
       <c r="F63" t="s">
-        <v>109</v>
+        <v>58</v>
       </c>
       <c r="G63" t="s">
-        <v>35</v>
+        <v>64</v>
       </c>
       <c r="H63" t="s">
         <v>18</v>
@@ -2796,54 +2802,54 @@
     </row>
     <row r="64" spans="1:9" ht="15">
       <c r="A64" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B64" t="s">
-        <v>12</v>
+        <v>54</v>
       </c>
       <c r="C64" t="s">
-        <v>13</v>
+        <v>90</v>
       </c>
       <c r="D64" t="s">
-        <v>40</v>
+        <v>85</v>
       </c>
       <c r="E64" t="s">
-        <v>99</v>
+        <v>118</v>
       </c>
       <c r="F64" t="s">
-        <v>68</v>
+        <v>111</v>
       </c>
       <c r="G64" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="H64" t="s">
         <v>18</v>
       </c>
       <c r="I64" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="65" spans="1:9" ht="15">
       <c r="A65" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B65" t="s">
-        <v>20</v>
+        <v>54</v>
       </c>
       <c r="C65" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D65" t="s">
-        <v>56</v>
+        <v>116</v>
       </c>
       <c r="E65" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="F65" t="s">
-        <v>114</v>
+        <v>97</v>
       </c>
       <c r="G65" t="s">
-        <v>98</v>
+        <v>117</v>
       </c>
       <c r="H65" t="s">
         <v>18</v>
@@ -2854,25 +2860,25 @@
     </row>
     <row r="66" spans="1:9" ht="15">
       <c r="A66" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B66" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="C66" t="s">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="D66" t="s">
-        <v>40</v>
+        <v>62</v>
       </c>
       <c r="E66" t="s">
-        <v>30</v>
+        <v>63</v>
       </c>
       <c r="F66" t="s">
-        <v>68</v>
+        <v>58</v>
       </c>
       <c r="G66" t="s">
-        <v>100</v>
+        <v>64</v>
       </c>
       <c r="H66" t="s">
         <v>18</v>
@@ -2883,68 +2889,68 @@
     </row>
     <row r="67" spans="1:9" ht="15">
       <c r="A67" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B67" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="C67" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D67" t="s">
-        <v>88</v>
+        <v>85</v>
       </c>
       <c r="E67" t="s">
         <v>89</v>
       </c>
       <c r="F67" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="G67" t="s">
-        <v>116</v>
+        <v>49</v>
       </c>
       <c r="H67" t="s">
         <v>18</v>
       </c>
       <c r="I67" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="68" spans="1:9" ht="15">
       <c r="A68" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B68" t="s">
-        <v>21</v>
+        <v>61</v>
       </c>
       <c r="C68" t="s">
         <v>24</v>
       </c>
       <c r="D68" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="E68" t="s">
-        <v>47</v>
+        <v>26</v>
       </c>
       <c r="F68" t="s">
-        <v>48</v>
+        <v>109</v>
       </c>
       <c r="G68" t="s">
-        <v>17</v>
+        <v>35</v>
       </c>
       <c r="H68" t="s">
         <v>18</v>
       </c>
       <c r="I68" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="69" spans="1:9" ht="15">
       <c r="A69" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B69" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="C69" t="s">
         <v>13</v>
@@ -2953,7 +2959,7 @@
         <v>40</v>
       </c>
       <c r="E69" t="s">
-        <v>30</v>
+        <v>99</v>
       </c>
       <c r="F69" t="s">
         <v>68</v>
@@ -2970,25 +2976,25 @@
     </row>
     <row r="70" spans="1:9" ht="15">
       <c r="A70" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B70" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C70" t="s">
         <v>81</v>
       </c>
       <c r="D70" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="E70" t="s">
-        <v>117</v>
+        <v>50</v>
       </c>
       <c r="F70" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="G70" t="s">
-        <v>118</v>
+        <v>98</v>
       </c>
       <c r="H70" t="s">
         <v>18</v>
@@ -2999,25 +3005,25 @@
     </row>
     <row r="71" spans="1:9" ht="15">
       <c r="A71" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B71" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C71" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D71" t="s">
-        <v>96</v>
+        <v>40</v>
       </c>
       <c r="E71" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F71" t="s">
-        <v>114</v>
+        <v>68</v>
       </c>
       <c r="G71" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="H71" t="s">
         <v>18</v>
@@ -3028,25 +3034,25 @@
     </row>
     <row r="72" spans="1:9" ht="15">
       <c r="A72" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B72" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C72" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D72" t="s">
-        <v>40</v>
+        <v>88</v>
       </c>
       <c r="E72" t="s">
-        <v>30</v>
+        <v>89</v>
       </c>
       <c r="F72" t="s">
-        <v>16</v>
+        <v>111</v>
       </c>
       <c r="G72" t="s">
-        <v>100</v>
+        <v>121</v>
       </c>
       <c r="H72" t="s">
         <v>18</v>
@@ -3057,83 +3063,83 @@
     </row>
     <row r="73" spans="1:9" ht="15">
       <c r="A73" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B73" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C73" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D73" t="s">
-        <v>119</v>
+        <v>96</v>
       </c>
       <c r="E73" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="F73" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="G73" t="s">
-        <v>120</v>
+        <v>17</v>
       </c>
       <c r="H73" t="s">
         <v>18</v>
       </c>
       <c r="I73" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="15">
       <c r="A74" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B74" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C74" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D74" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="E74" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F74" t="s">
-        <v>48</v>
+        <v>68</v>
       </c>
       <c r="G74" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="H74" t="s">
         <v>18</v>
       </c>
       <c r="I74" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="75" spans="1:9" ht="15">
       <c r="A75" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B75" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C75" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D75" t="s">
-        <v>40</v>
+        <v>46</v>
       </c>
       <c r="E75" t="s">
-        <v>30</v>
+        <v>118</v>
       </c>
       <c r="F75" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="G75" t="s">
-        <v>100</v>
+        <v>122</v>
       </c>
       <c r="H75" t="s">
         <v>18</v>
@@ -3144,25 +3150,25 @@
     </row>
     <row r="76" spans="1:9" ht="15">
       <c r="A76" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B76" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C76" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D76" t="s">
-        <v>85</v>
+        <v>96</v>
       </c>
       <c r="E76" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="F76" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="G76" t="s">
-        <v>116</v>
+        <v>98</v>
       </c>
       <c r="H76" t="s">
         <v>18</v>
@@ -3173,54 +3179,54 @@
     </row>
     <row r="77" spans="1:9" ht="15">
       <c r="A77" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B77" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C77" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D77" t="s">
-        <v>91</v>
+        <v>40</v>
       </c>
       <c r="E77" t="s">
-        <v>47</v>
+        <v>30</v>
       </c>
       <c r="F77" t="s">
-        <v>48</v>
+        <v>16</v>
       </c>
       <c r="G77" t="s">
-        <v>17</v>
+        <v>100</v>
       </c>
       <c r="H77" t="s">
         <v>18</v>
       </c>
       <c r="I77" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="15">
       <c r="A78" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B78" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C78" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D78" t="s">
-        <v>40</v>
+        <v>123</v>
       </c>
       <c r="E78" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="F78" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="G78" t="s">
-        <v>100</v>
+        <v>124</v>
       </c>
       <c r="H78" t="s">
         <v>18</v>
@@ -3231,54 +3237,54 @@
     </row>
     <row r="79" spans="1:9" ht="15">
       <c r="A79" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B79" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C79" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D79" t="s">
-        <v>121</v>
+        <v>91</v>
       </c>
       <c r="E79" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="F79" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="G79" t="s">
-        <v>120</v>
+        <v>17</v>
       </c>
       <c r="H79" t="s">
         <v>18</v>
       </c>
       <c r="I79" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="15">
       <c r="A80" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B80" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C80" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D80" t="s">
-        <v>111</v>
+        <v>40</v>
       </c>
       <c r="E80" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F80" t="s">
-        <v>122</v>
+        <v>16</v>
       </c>
       <c r="G80" t="s">
-        <v>35</v>
+        <v>100</v>
       </c>
       <c r="H80" t="s">
         <v>18</v>
@@ -3289,25 +3295,25 @@
     </row>
     <row r="81" spans="1:9" ht="15">
       <c r="A81" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B81" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C81" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D81" t="s">
-        <v>111</v>
+        <v>85</v>
       </c>
       <c r="E81" t="s">
-        <v>123</v>
+        <v>89</v>
       </c>
       <c r="F81" t="s">
-        <v>124</v>
+        <v>68</v>
       </c>
       <c r="G81" t="s">
-        <v>125</v>
+        <v>121</v>
       </c>
       <c r="H81" t="s">
         <v>18</v>
@@ -3318,30 +3324,175 @@
     </row>
     <row r="82" spans="1:9" ht="15">
       <c r="A82" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B82" t="s">
-        <v>61</v>
+        <v>44</v>
       </c>
       <c r="C82" t="s">
         <v>24</v>
       </c>
       <c r="D82" t="s">
-        <v>111</v>
+        <v>91</v>
       </c>
       <c r="E82" t="s">
-        <v>123</v>
+        <v>47</v>
       </c>
       <c r="F82" t="s">
+        <v>48</v>
+      </c>
+      <c r="G82" t="s">
+        <v>17</v>
+      </c>
+      <c r="H82" t="s">
+        <v>18</v>
+      </c>
+      <c r="I82" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="15">
+      <c r="A83" t="s">
+        <v>119</v>
+      </c>
+      <c r="B83" t="s">
+        <v>44</v>
+      </c>
+      <c r="C83" t="s">
+        <v>13</v>
+      </c>
+      <c r="D83" t="s">
+        <v>40</v>
+      </c>
+      <c r="E83" t="s">
+        <v>50</v>
+      </c>
+      <c r="F83" t="s">
+        <v>16</v>
+      </c>
+      <c r="G83" t="s">
+        <v>100</v>
+      </c>
+      <c r="H83" t="s">
+        <v>18</v>
+      </c>
+      <c r="I83" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="15">
+      <c r="A84" t="s">
+        <v>119</v>
+      </c>
+      <c r="B84" t="s">
+        <v>53</v>
+      </c>
+      <c r="C84" t="s">
+        <v>81</v>
+      </c>
+      <c r="D84" t="s">
+        <v>114</v>
+      </c>
+      <c r="E84" t="s">
+        <v>89</v>
+      </c>
+      <c r="F84" t="s">
+        <v>68</v>
+      </c>
+      <c r="G84" t="s">
         <v>124</v>
       </c>
-      <c r="G82" t="s">
+      <c r="H84" t="s">
+        <v>18</v>
+      </c>
+      <c r="I84" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="15">
+      <c r="A85" t="s">
+        <v>119</v>
+      </c>
+      <c r="B85" t="s">
+        <v>53</v>
+      </c>
+      <c r="C85" t="s">
+        <v>24</v>
+      </c>
+      <c r="D85" t="s">
+        <v>116</v>
+      </c>
+      <c r="E85" t="s">
+        <v>50</v>
+      </c>
+      <c r="F85" t="s">
         <v>125</v>
       </c>
-      <c r="H82" t="s">
-        <v>18</v>
-      </c>
-      <c r="I82" t="s">
+      <c r="G85" t="s">
+        <v>35</v>
+      </c>
+      <c r="H85" t="s">
+        <v>18</v>
+      </c>
+      <c r="I85" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="15">
+      <c r="A86" t="s">
+        <v>119</v>
+      </c>
+      <c r="B86" t="s">
+        <v>54</v>
+      </c>
+      <c r="C86" t="s">
+        <v>24</v>
+      </c>
+      <c r="D86" t="s">
+        <v>116</v>
+      </c>
+      <c r="E86" t="s">
+        <v>126</v>
+      </c>
+      <c r="F86" t="s">
+        <v>127</v>
+      </c>
+      <c r="G86" t="s">
+        <v>128</v>
+      </c>
+      <c r="H86" t="s">
+        <v>18</v>
+      </c>
+      <c r="I86" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="15">
+      <c r="A87" t="s">
+        <v>119</v>
+      </c>
+      <c r="B87" t="s">
+        <v>61</v>
+      </c>
+      <c r="C87" t="s">
+        <v>24</v>
+      </c>
+      <c r="D87" t="s">
+        <v>116</v>
+      </c>
+      <c r="E87" t="s">
+        <v>126</v>
+      </c>
+      <c r="F87" t="s">
+        <v>127</v>
+      </c>
+      <c r="G87" t="s">
+        <v>128</v>
+      </c>
+      <c r="H87" t="s">
+        <v>18</v>
+      </c>
+      <c r="I87" t="s">
         <v>29</v>
       </c>
     </row>
@@ -3353,8 +3504,8 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{b1b049b6-5e1c-4221-9ea7-9dcb0b353103}">
-  <dimension ref="A1:F17"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{04eb977a-c1db-4a18-8743-599b6112ef49}">
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
@@ -3370,13 +3521,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -3390,16 +3541,16 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -3410,16 +3561,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E3" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -3430,16 +3581,16 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E4" t="s">
-        <v>134</v>
+        <v>112</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -3450,16 +3601,16 @@
         <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C5" t="s">
         <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E5" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -3470,16 +3621,16 @@
         <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E6" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -3490,13 +3641,13 @@
         <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C7" t="s">
         <v>81</v>
       </c>
       <c r="D7" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E7" t="s">
         <v>28</v>
@@ -3510,13 +3661,13 @@
         <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E8" t="s">
         <v>98</v>
@@ -3530,16 +3681,16 @@
         <v>95</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C9" t="s">
         <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="E9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -3550,16 +3701,16 @@
         <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C10" t="s">
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E10" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -3570,16 +3721,16 @@
         <v>95</v>
       </c>
       <c r="B11" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="E11" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -3587,19 +3738,19 @@
     </row>
     <row r="12" spans="1:6" ht="15">
       <c r="A12" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>137</v>
       </c>
       <c r="C12" t="s">
-        <v>81</v>
+        <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E12" t="s">
-        <v>149</v>
+        <v>35</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -3607,19 +3758,19 @@
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B13" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D13" t="s">
-        <v>130</v>
+        <v>150</v>
       </c>
       <c r="E13" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -3627,7 +3778,7 @@
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B14" t="s">
         <v>146</v>
@@ -3636,10 +3787,10 @@
         <v>13</v>
       </c>
       <c r="D14" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E14" t="s">
-        <v>75</v>
+        <v>152</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -3647,19 +3798,19 @@
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B15" t="s">
+        <v>148</v>
+      </c>
+      <c r="C15" t="s">
+        <v>13</v>
+      </c>
+      <c r="D15" t="s">
         <v>133</v>
       </c>
-      <c r="C15" t="s">
-        <v>81</v>
-      </c>
-      <c r="D15" t="s">
-        <v>141</v>
-      </c>
       <c r="E15" t="s">
-        <v>151</v>
+        <v>75</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -3667,19 +3818,19 @@
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B16" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D16" t="s">
         <v>143</v>
       </c>
       <c r="E16" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -3687,21 +3838,41 @@
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="B17" t="s">
-        <v>153</v>
+        <v>136</v>
       </c>
       <c r="C17" t="s">
         <v>24</v>
       </c>
       <c r="D17" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="E17" t="s">
-        <v>112</v>
+        <v>154</v>
       </c>
       <c r="F17" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" ht="15">
+      <c r="A18" t="s">
+        <v>119</v>
+      </c>
+      <c r="B18" t="s">
+        <v>155</v>
+      </c>
+      <c r="C18" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" t="s">
+        <v>145</v>
+      </c>
+      <c r="E18" t="s">
+        <v>117</v>
+      </c>
+      <c r="F18" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update substitutions September 10 afternoon
</commit_message>
<xml_diff>
--- a/InformacjeOZastepstwach.xlsx
+++ b/InformacjeOZastepstwach.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="893" uniqueCount="156">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="962" uniqueCount="164">
   <si>
     <t>Rok szkolny: 2026/2027</t>
   </si>
@@ -319,67 +319,82 @@
     <t>Jastrzębska-Majtyka Agnieszka</t>
   </si>
   <si>
+    <t>Kończyńska Małgorzata</t>
+  </si>
+  <si>
+    <t>5TFB</t>
+  </si>
+  <si>
+    <t>2CA|CH</t>
+  </si>
+  <si>
+    <t>Wychowanie fizyczne</t>
+  </si>
+  <si>
+    <t>22</t>
+  </si>
+  <si>
+    <t>Pietrycha Małgorzata</t>
+  </si>
+  <si>
+    <t>2CA|DZ</t>
+  </si>
+  <si>
+    <t>1FA|gr1</t>
+  </si>
+  <si>
+    <t>1FA|gr2</t>
+  </si>
+  <si>
+    <t>32</t>
+  </si>
+  <si>
+    <t>2WA</t>
+  </si>
+  <si>
+    <t>28</t>
+  </si>
+  <si>
+    <t>Wójcik Kamil</t>
+  </si>
+  <si>
+    <t>26</t>
+  </si>
+  <si>
+    <t>1FA</t>
+  </si>
+  <si>
+    <t>Filipek Anna</t>
+  </si>
+  <si>
+    <t>1TFB</t>
+  </si>
+  <si>
+    <t>Danielewski Paweł</t>
+  </si>
+  <si>
+    <t>Chemia</t>
+  </si>
+  <si>
+    <t>Ostrowska Ewa</t>
+  </si>
+  <si>
+    <t>2CB</t>
+  </si>
+  <si>
+    <t>29</t>
+  </si>
+  <si>
+    <t>1K</t>
+  </si>
+  <si>
+    <t>11.09.2026</t>
+  </si>
+  <si>
     <t>Rozwój kompetencji zawodowych - dekoracje w cukiernictwie</t>
   </si>
   <si>
-    <t>Kończyńska Małgorzata</t>
-  </si>
-  <si>
-    <t>5TFB</t>
-  </si>
-  <si>
-    <t>2CA|CH</t>
-  </si>
-  <si>
-    <t>Wychowanie fizyczne</t>
-  </si>
-  <si>
-    <t>22</t>
-  </si>
-  <si>
-    <t>Pietrycha Małgorzata</t>
-  </si>
-  <si>
-    <t>2CA|DZ</t>
-  </si>
-  <si>
-    <t>1FA|gr1</t>
-  </si>
-  <si>
-    <t>1FA|gr2</t>
-  </si>
-  <si>
-    <t>32</t>
-  </si>
-  <si>
-    <t>2WA</t>
-  </si>
-  <si>
-    <t>28</t>
-  </si>
-  <si>
-    <t>Wójcik Kamil</t>
-  </si>
-  <si>
-    <t>26</t>
-  </si>
-  <si>
-    <t>1FA</t>
-  </si>
-  <si>
-    <t>Filipek Anna</t>
-  </si>
-  <si>
-    <t>1TFB</t>
-  </si>
-  <si>
-    <t>Danielewski Paweł</t>
-  </si>
-  <si>
-    <t>Chemia</t>
-  </si>
-  <si>
-    <t>11.09.2026</t>
+    <t>Hudziec Agnieszka</t>
   </si>
   <si>
     <t>3</t>
@@ -388,7 +403,7 @@
     <t>Małecka Barbara</t>
   </si>
   <si>
-    <t>Hudziec Agnieszka</t>
+    <t>1TH</t>
   </si>
   <si>
     <t>1TFA</t>
@@ -397,6 +412,12 @@
     <t>Sałdyka Karolina</t>
   </si>
   <si>
+    <t>3FB</t>
+  </si>
+  <si>
+    <t>1TFH</t>
+  </si>
+  <si>
     <t>43</t>
   </si>
   <si>
@@ -473,6 +494,9 @@
   </si>
   <si>
     <t>piętro_2</t>
+  </si>
+  <si>
+    <t>Świerzewicz Katarzyna</t>
   </si>
   <si>
     <t>Karczmarz Aleksandra</t>
@@ -937,7 +961,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{f5905cba-1004-41ce-85e8-c077faefae63}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{7b69b720-263f-409a-8ace-71751a1182b4}">
   <dimension ref="A1:A2"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
@@ -958,8 +982,8 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{a4da12a8-2b8c-4c9b-96fe-b6984f3133b1}">
-  <dimension ref="A1:I87"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{65802c7f-f101-4504-9092-87d613bbd669}">
+  <dimension ref="A1:I94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
@@ -2176,13 +2200,13 @@
         <v>14</v>
       </c>
       <c r="E42" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="F42" t="s">
         <v>68</v>
       </c>
       <c r="G42" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H42" t="s">
         <v>18</v>
@@ -2202,7 +2226,7 @@
         <v>81</v>
       </c>
       <c r="D43" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E43" t="s">
         <v>82</v>
@@ -2263,13 +2287,13 @@
         <v>14</v>
       </c>
       <c r="E45" t="s">
-        <v>99</v>
+        <v>30</v>
       </c>
       <c r="F45" t="s">
         <v>68</v>
       </c>
       <c r="G45" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H45" t="s">
         <v>18</v>
@@ -2289,7 +2313,7 @@
         <v>81</v>
       </c>
       <c r="D46" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E46" t="s">
         <v>82</v>
@@ -2347,16 +2371,16 @@
         <v>13</v>
       </c>
       <c r="D48" t="s">
+        <v>101</v>
+      </c>
+      <c r="E48" t="s">
         <v>102</v>
       </c>
-      <c r="E48" t="s">
+      <c r="F48" t="s">
         <v>103</v>
       </c>
-      <c r="F48" t="s">
+      <c r="G48" t="s">
         <v>104</v>
-      </c>
-      <c r="G48" t="s">
-        <v>105</v>
       </c>
       <c r="H48" t="s">
         <v>18</v>
@@ -2376,16 +2400,16 @@
         <v>13</v>
       </c>
       <c r="D49" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E49" t="s">
+        <v>102</v>
+      </c>
+      <c r="F49" t="s">
         <v>103</v>
       </c>
-      <c r="F49" t="s">
+      <c r="G49" t="s">
         <v>104</v>
-      </c>
-      <c r="G49" t="s">
-        <v>105</v>
       </c>
       <c r="H49" t="s">
         <v>18</v>
@@ -2405,16 +2429,16 @@
         <v>81</v>
       </c>
       <c r="D50" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E50" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F50" t="s">
         <v>68</v>
       </c>
       <c r="G50" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H50" t="s">
         <v>18</v>
@@ -2434,16 +2458,16 @@
         <v>81</v>
       </c>
       <c r="D51" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E51" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F51" t="s">
         <v>68</v>
       </c>
       <c r="G51" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="H51" t="s">
         <v>18</v>
@@ -2498,10 +2522,10 @@
         <v>30</v>
       </c>
       <c r="F53" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G53" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H53" t="s">
         <v>18</v>
@@ -2521,16 +2545,16 @@
         <v>90</v>
       </c>
       <c r="D54" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E54" t="s">
         <v>50</v>
       </c>
       <c r="F54" t="s">
+        <v>110</v>
+      </c>
+      <c r="G54" t="s">
         <v>111</v>
-      </c>
-      <c r="G54" t="s">
-        <v>112</v>
       </c>
       <c r="H54" t="s">
         <v>18</v>
@@ -2585,10 +2609,10 @@
         <v>30</v>
       </c>
       <c r="F56" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="G56" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H56" t="s">
         <v>18</v>
@@ -2608,16 +2632,16 @@
         <v>90</v>
       </c>
       <c r="D57" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E57" t="s">
         <v>82</v>
       </c>
       <c r="F57" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G57" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="H57" t="s">
         <v>18</v>
@@ -2704,7 +2728,7 @@
         <v>68</v>
       </c>
       <c r="G60" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H60" t="s">
         <v>18</v>
@@ -2753,16 +2777,16 @@
         <v>90</v>
       </c>
       <c r="D62" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E62" t="s">
         <v>47</v>
       </c>
       <c r="F62" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G62" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H62" t="s">
         <v>18</v>
@@ -2814,10 +2838,10 @@
         <v>85</v>
       </c>
       <c r="E64" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F64" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G64" t="s">
         <v>49</v>
@@ -2840,7 +2864,7 @@
         <v>24</v>
       </c>
       <c r="D65" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E65" t="s">
         <v>47</v>
@@ -2849,7 +2873,7 @@
         <v>97</v>
       </c>
       <c r="G65" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="H65" t="s">
         <v>18</v>
@@ -2904,7 +2928,7 @@
         <v>89</v>
       </c>
       <c r="F67" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="G67" t="s">
         <v>49</v>
@@ -2933,7 +2957,7 @@
         <v>26</v>
       </c>
       <c r="F68" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="G68" t="s">
         <v>35</v>
@@ -2947,68 +2971,68 @@
     </row>
     <row r="69" spans="1:9" ht="15">
       <c r="A69" t="s">
+        <v>95</v>
+      </c>
+      <c r="B69" t="s">
+        <v>78</v>
+      </c>
+      <c r="C69" t="s">
+        <v>118</v>
+      </c>
+      <c r="D69" t="s">
         <v>119</v>
       </c>
-      <c r="B69" t="s">
-        <v>12</v>
-      </c>
-      <c r="C69" t="s">
-        <v>13</v>
-      </c>
-      <c r="D69" t="s">
-        <v>40</v>
-      </c>
       <c r="E69" t="s">
-        <v>99</v>
+        <v>63</v>
       </c>
       <c r="F69" t="s">
-        <v>68</v>
+        <v>120</v>
       </c>
       <c r="G69" t="s">
-        <v>100</v>
+        <v>49</v>
       </c>
       <c r="H69" t="s">
         <v>18</v>
       </c>
       <c r="I69" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="70" spans="1:9" ht="15">
       <c r="A70" t="s">
-        <v>119</v>
+        <v>95</v>
       </c>
       <c r="B70" t="s">
-        <v>20</v>
+        <v>65</v>
       </c>
       <c r="C70" t="s">
-        <v>81</v>
+        <v>118</v>
       </c>
       <c r="D70" t="s">
-        <v>56</v>
+        <v>121</v>
       </c>
       <c r="E70" t="s">
-        <v>50</v>
+        <v>63</v>
       </c>
       <c r="F70" t="s">
         <v>120</v>
       </c>
       <c r="G70" t="s">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="H70" t="s">
         <v>18</v>
       </c>
       <c r="I70" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="71" spans="1:9" ht="15">
       <c r="A71" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B71" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="C71" t="s">
         <v>13</v>
@@ -3017,13 +3041,13 @@
         <v>40</v>
       </c>
       <c r="E71" t="s">
-        <v>30</v>
+        <v>123</v>
       </c>
       <c r="F71" t="s">
         <v>68</v>
       </c>
       <c r="G71" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H71" t="s">
         <v>18</v>
@@ -3034,68 +3058,68 @@
     </row>
     <row r="72" spans="1:9" ht="15">
       <c r="A72" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B72" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C72" t="s">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="D72" t="s">
         <v>88</v>
       </c>
       <c r="E72" t="s">
-        <v>89</v>
+        <v>117</v>
       </c>
       <c r="F72" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="G72" t="s">
-        <v>121</v>
+        <v>17</v>
       </c>
       <c r="H72" t="s">
         <v>18</v>
       </c>
       <c r="I72" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="73" spans="1:9" ht="15">
       <c r="A73" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B73" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C73" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D73" t="s">
-        <v>96</v>
+        <v>56</v>
       </c>
       <c r="E73" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="F73" t="s">
-        <v>48</v>
+        <v>125</v>
       </c>
       <c r="G73" t="s">
-        <v>17</v>
+        <v>98</v>
       </c>
       <c r="H73" t="s">
         <v>18</v>
       </c>
       <c r="I73" t="s">
-        <v>19</v>
+        <v>29</v>
       </c>
     </row>
     <row r="74" spans="1:9" ht="15">
       <c r="A74" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B74" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C74" t="s">
         <v>13</v>
@@ -3110,7 +3134,7 @@
         <v>68</v>
       </c>
       <c r="G74" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="H74" t="s">
         <v>18</v>
@@ -3121,54 +3145,54 @@
     </row>
     <row r="75" spans="1:9" ht="15">
       <c r="A75" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B75" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C75" t="s">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="D75" t="s">
-        <v>46</v>
+        <v>121</v>
       </c>
       <c r="E75" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F75" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="G75" t="s">
-        <v>122</v>
+        <v>17</v>
       </c>
       <c r="H75" t="s">
         <v>18</v>
       </c>
       <c r="I75" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="76" spans="1:9" ht="15">
       <c r="A76" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B76" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C76" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D76" t="s">
-        <v>96</v>
+        <v>88</v>
       </c>
       <c r="E76" t="s">
-        <v>47</v>
+        <v>89</v>
       </c>
       <c r="F76" t="s">
-        <v>120</v>
+        <v>110</v>
       </c>
       <c r="G76" t="s">
-        <v>98</v>
+        <v>126</v>
       </c>
       <c r="H76" t="s">
         <v>18</v>
@@ -3179,54 +3203,54 @@
     </row>
     <row r="77" spans="1:9" ht="15">
       <c r="A77" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B77" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C77" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D77" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="E77" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="F77" t="s">
-        <v>16</v>
+        <v>48</v>
       </c>
       <c r="G77" t="s">
-        <v>100</v>
+        <v>17</v>
       </c>
       <c r="H77" t="s">
         <v>18</v>
       </c>
       <c r="I77" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="78" spans="1:9" ht="15">
       <c r="A78" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B78" t="s">
-        <v>31</v>
+        <v>21</v>
       </c>
       <c r="C78" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D78" t="s">
-        <v>123</v>
+        <v>40</v>
       </c>
       <c r="E78" t="s">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="F78" t="s">
         <v>68</v>
       </c>
       <c r="G78" t="s">
-        <v>124</v>
+        <v>99</v>
       </c>
       <c r="H78" t="s">
         <v>18</v>
@@ -3237,54 +3261,54 @@
     </row>
     <row r="79" spans="1:9" ht="15">
       <c r="A79" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B79" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C79" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D79" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="E79" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="F79" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="G79" t="s">
-        <v>17</v>
+        <v>60</v>
       </c>
       <c r="H79" t="s">
         <v>18</v>
       </c>
       <c r="I79" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="80" spans="1:9" ht="15">
       <c r="A80" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B80" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="C80" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="D80" t="s">
-        <v>40</v>
+        <v>96</v>
       </c>
       <c r="E80" t="s">
-        <v>30</v>
+        <v>47</v>
       </c>
       <c r="F80" t="s">
-        <v>16</v>
+        <v>125</v>
       </c>
       <c r="G80" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="H80" t="s">
         <v>18</v>
@@ -3295,25 +3319,25 @@
     </row>
     <row r="81" spans="1:9" ht="15">
       <c r="A81" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B81" t="s">
-        <v>44</v>
+        <v>23</v>
       </c>
       <c r="C81" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D81" t="s">
-        <v>85</v>
+        <v>40</v>
       </c>
       <c r="E81" t="s">
-        <v>89</v>
+        <v>30</v>
       </c>
       <c r="F81" t="s">
         <v>68</v>
       </c>
       <c r="G81" t="s">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="H81" t="s">
         <v>18</v>
@@ -3324,22 +3348,22 @@
     </row>
     <row r="82" spans="1:9" ht="15">
       <c r="A82" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B82" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C82" t="s">
-        <v>24</v>
+        <v>124</v>
       </c>
       <c r="D82" t="s">
-        <v>91</v>
+        <v>127</v>
       </c>
       <c r="E82" t="s">
-        <v>47</v>
+        <v>117</v>
       </c>
       <c r="F82" t="s">
-        <v>48</v>
+        <v>112</v>
       </c>
       <c r="G82" t="s">
         <v>17</v>
@@ -3353,25 +3377,25 @@
     </row>
     <row r="83" spans="1:9" ht="15">
       <c r="A83" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B83" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="C83" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D83" t="s">
-        <v>40</v>
+        <v>128</v>
       </c>
       <c r="E83" t="s">
-        <v>50</v>
+        <v>89</v>
       </c>
       <c r="F83" t="s">
-        <v>16</v>
+        <v>68</v>
       </c>
       <c r="G83" t="s">
-        <v>100</v>
+        <v>129</v>
       </c>
       <c r="H83" t="s">
         <v>18</v>
@@ -3382,54 +3406,54 @@
     </row>
     <row r="84" spans="1:9" ht="15">
       <c r="A84" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B84" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C84" t="s">
-        <v>81</v>
+        <v>24</v>
       </c>
       <c r="D84" t="s">
-        <v>114</v>
+        <v>91</v>
       </c>
       <c r="E84" t="s">
-        <v>89</v>
+        <v>47</v>
       </c>
       <c r="F84" t="s">
-        <v>68</v>
+        <v>48</v>
       </c>
       <c r="G84" t="s">
-        <v>124</v>
+        <v>17</v>
       </c>
       <c r="H84" t="s">
         <v>18</v>
       </c>
       <c r="I84" t="s">
-        <v>29</v>
+        <v>19</v>
       </c>
     </row>
     <row r="85" spans="1:9" ht="15">
       <c r="A85" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B85" t="s">
-        <v>53</v>
+        <v>31</v>
       </c>
       <c r="C85" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="D85" t="s">
-        <v>116</v>
+        <v>40</v>
       </c>
       <c r="E85" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="F85" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="G85" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="H85" t="s">
         <v>18</v>
@@ -3440,59 +3464,262 @@
     </row>
     <row r="86" spans="1:9" ht="15">
       <c r="A86" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B86" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
       <c r="C86" t="s">
-        <v>24</v>
+        <v>124</v>
       </c>
       <c r="D86" t="s">
-        <v>116</v>
+        <v>130</v>
       </c>
       <c r="E86" t="s">
-        <v>126</v>
+        <v>36</v>
       </c>
       <c r="F86" t="s">
-        <v>127</v>
+        <v>37</v>
       </c>
       <c r="G86" t="s">
-        <v>128</v>
+        <v>38</v>
       </c>
       <c r="H86" t="s">
         <v>18</v>
       </c>
       <c r="I86" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
     </row>
     <row r="87" spans="1:9" ht="15">
       <c r="A87" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B87" t="s">
+        <v>44</v>
+      </c>
+      <c r="C87" t="s">
+        <v>81</v>
+      </c>
+      <c r="D87" t="s">
+        <v>85</v>
+      </c>
+      <c r="E87" t="s">
+        <v>89</v>
+      </c>
+      <c r="F87" t="s">
+        <v>68</v>
+      </c>
+      <c r="G87" t="s">
+        <v>126</v>
+      </c>
+      <c r="H87" t="s">
+        <v>18</v>
+      </c>
+      <c r="I87" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="15">
+      <c r="A88" t="s">
+        <v>122</v>
+      </c>
+      <c r="B88" t="s">
+        <v>44</v>
+      </c>
+      <c r="C88" t="s">
+        <v>24</v>
+      </c>
+      <c r="D88" t="s">
+        <v>91</v>
+      </c>
+      <c r="E88" t="s">
+        <v>47</v>
+      </c>
+      <c r="F88" t="s">
+        <v>48</v>
+      </c>
+      <c r="G88" t="s">
+        <v>17</v>
+      </c>
+      <c r="H88" t="s">
+        <v>18</v>
+      </c>
+      <c r="I88" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="15">
+      <c r="A89" t="s">
+        <v>122</v>
+      </c>
+      <c r="B89" t="s">
+        <v>44</v>
+      </c>
+      <c r="C89" t="s">
+        <v>13</v>
+      </c>
+      <c r="D89" t="s">
+        <v>40</v>
+      </c>
+      <c r="E89" t="s">
+        <v>50</v>
+      </c>
+      <c r="F89" t="s">
+        <v>112</v>
+      </c>
+      <c r="G89" t="s">
+        <v>99</v>
+      </c>
+      <c r="H89" t="s">
+        <v>18</v>
+      </c>
+      <c r="I89" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="15">
+      <c r="A90" t="s">
+        <v>122</v>
+      </c>
+      <c r="B90" t="s">
+        <v>53</v>
+      </c>
+      <c r="C90" t="s">
+        <v>124</v>
+      </c>
+      <c r="D90" t="s">
+        <v>131</v>
+      </c>
+      <c r="E90" t="s">
+        <v>36</v>
+      </c>
+      <c r="F90" t="s">
+        <v>37</v>
+      </c>
+      <c r="G90" t="s">
+        <v>38</v>
+      </c>
+      <c r="H90" t="s">
+        <v>18</v>
+      </c>
+      <c r="I90" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="15">
+      <c r="A91" t="s">
+        <v>122</v>
+      </c>
+      <c r="B91" t="s">
+        <v>53</v>
+      </c>
+      <c r="C91" t="s">
+        <v>81</v>
+      </c>
+      <c r="D91" t="s">
+        <v>113</v>
+      </c>
+      <c r="E91" t="s">
+        <v>89</v>
+      </c>
+      <c r="F91" t="s">
+        <v>68</v>
+      </c>
+      <c r="G91" t="s">
+        <v>129</v>
+      </c>
+      <c r="H91" t="s">
+        <v>18</v>
+      </c>
+      <c r="I91" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="15">
+      <c r="A92" t="s">
+        <v>122</v>
+      </c>
+      <c r="B92" t="s">
+        <v>53</v>
+      </c>
+      <c r="C92" t="s">
+        <v>24</v>
+      </c>
+      <c r="D92" t="s">
+        <v>115</v>
+      </c>
+      <c r="E92" t="s">
+        <v>50</v>
+      </c>
+      <c r="F92" t="s">
+        <v>132</v>
+      </c>
+      <c r="G92" t="s">
+        <v>35</v>
+      </c>
+      <c r="H92" t="s">
+        <v>18</v>
+      </c>
+      <c r="I92" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="15">
+      <c r="A93" t="s">
+        <v>122</v>
+      </c>
+      <c r="B93" t="s">
+        <v>54</v>
+      </c>
+      <c r="C93" t="s">
+        <v>24</v>
+      </c>
+      <c r="D93" t="s">
+        <v>115</v>
+      </c>
+      <c r="E93" t="s">
+        <v>133</v>
+      </c>
+      <c r="F93" t="s">
+        <v>134</v>
+      </c>
+      <c r="G93" t="s">
+        <v>135</v>
+      </c>
+      <c r="H93" t="s">
+        <v>18</v>
+      </c>
+      <c r="I93" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="15">
+      <c r="A94" t="s">
+        <v>122</v>
+      </c>
+      <c r="B94" t="s">
         <v>61</v>
       </c>
-      <c r="C87" t="s">
+      <c r="C94" t="s">
         <v>24</v>
       </c>
-      <c r="D87" t="s">
-        <v>116</v>
-      </c>
-      <c r="E87" t="s">
-        <v>126</v>
-      </c>
-      <c r="F87" t="s">
-        <v>127</v>
-      </c>
-      <c r="G87" t="s">
-        <v>128</v>
-      </c>
-      <c r="H87" t="s">
-        <v>18</v>
-      </c>
-      <c r="I87" t="s">
+      <c r="D94" t="s">
+        <v>115</v>
+      </c>
+      <c r="E94" t="s">
+        <v>133</v>
+      </c>
+      <c r="F94" t="s">
+        <v>134</v>
+      </c>
+      <c r="G94" t="s">
+        <v>135</v>
+      </c>
+      <c r="H94" t="s">
+        <v>18</v>
+      </c>
+      <c r="I94" t="s">
         <v>29</v>
       </c>
     </row>
@@ -3504,13 +3731,13 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{04eb977a-c1db-4a18-8743-599b6112ef49}">
-  <dimension ref="A1:F18"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xr:uid="{5f4407a8-5b32-4469-94ef-9f5ffad6c2ad}">
+  <dimension ref="A1:F19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.4285714285714" customWidth="1"/>
     <col min="2" max="2" width="11.1428571428571" customWidth="1"/>
-    <col min="3" max="3" width="16" customWidth="1"/>
+    <col min="3" max="3" width="17.5714285714286" customWidth="1"/>
     <col min="4" max="4" width="35.1428571428571" customWidth="1"/>
     <col min="5" max="5" width="28.1428571428571" customWidth="1"/>
     <col min="6" max="6" width="9.28571428571429" customWidth="1"/>
@@ -3521,13 +3748,13 @@
         <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="E1" s="1" t="s">
         <v>8</v>
@@ -3541,16 +3768,16 @@
         <v>11</v>
       </c>
       <c r="B2" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C2" t="s">
         <v>13</v>
       </c>
       <c r="D2" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E2" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="F2" t="s">
         <v>18</v>
@@ -3561,16 +3788,16 @@
         <v>11</v>
       </c>
       <c r="B3" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C3" t="s">
         <v>24</v>
       </c>
       <c r="D3" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E3" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="F3" t="s">
         <v>18</v>
@@ -3581,16 +3808,16 @@
         <v>11</v>
       </c>
       <c r="B4" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C4" t="s">
         <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E4" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -3601,16 +3828,16 @@
         <v>71</v>
       </c>
       <c r="B5" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C5" t="s">
         <v>24</v>
       </c>
       <c r="D5" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="E5" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="F5" t="s">
         <v>18</v>
@@ -3621,16 +3848,16 @@
         <v>71</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="C6" t="s">
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="E6" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -3641,13 +3868,13 @@
         <v>80</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="C7" t="s">
         <v>81</v>
       </c>
       <c r="D7" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E7" t="s">
         <v>28</v>
@@ -3661,13 +3888,13 @@
         <v>95</v>
       </c>
       <c r="B8" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C8" t="s">
         <v>24</v>
       </c>
       <c r="D8" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E8" t="s">
         <v>98</v>
@@ -3681,16 +3908,16 @@
         <v>95</v>
       </c>
       <c r="B9" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C9" t="s">
         <v>81</v>
       </c>
       <c r="D9" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E9" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="F9" t="s">
         <v>18</v>
@@ -3701,16 +3928,16 @@
         <v>95</v>
       </c>
       <c r="B10" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C10" t="s">
         <v>13</v>
       </c>
       <c r="D10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E10" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -3721,16 +3948,16 @@
         <v>95</v>
       </c>
       <c r="B11" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="C11" t="s">
         <v>24</v>
       </c>
       <c r="D11" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="E11" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="F11" t="s">
         <v>18</v>
@@ -3741,13 +3968,13 @@
         <v>95</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
         <v>90</v>
       </c>
       <c r="D12" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="E12" t="s">
         <v>35</v>
@@ -3758,19 +3985,19 @@
     </row>
     <row r="13" spans="1:6" ht="15">
       <c r="A13" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>139</v>
       </c>
       <c r="C13" t="s">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="D13" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="E13" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="F13" t="s">
         <v>18</v>
@@ -3778,19 +4005,19 @@
     </row>
     <row r="14" spans="1:6" ht="15">
       <c r="A14" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B14" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="C14" t="s">
-        <v>13</v>
+        <v>81</v>
       </c>
       <c r="D14" t="s">
-        <v>133</v>
+        <v>157</v>
       </c>
       <c r="E14" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -3798,19 +4025,19 @@
     </row>
     <row r="15" spans="1:6" ht="15">
       <c r="A15" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="C15" t="s">
         <v>13</v>
       </c>
       <c r="D15" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="E15" t="s">
-        <v>75</v>
+        <v>160</v>
       </c>
       <c r="F15" t="s">
         <v>18</v>
@@ -3818,19 +4045,19 @@
     </row>
     <row r="16" spans="1:6" ht="15">
       <c r="A16" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B16" t="s">
-        <v>136</v>
+        <v>155</v>
       </c>
       <c r="C16" t="s">
-        <v>81</v>
+        <v>13</v>
       </c>
       <c r="D16" t="s">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="E16" t="s">
-        <v>153</v>
+        <v>75</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
@@ -3838,19 +4065,19 @@
     </row>
     <row r="17" spans="1:6" ht="15">
       <c r="A17" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B17" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>81</v>
       </c>
       <c r="D17" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="E17" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="F17" t="s">
         <v>18</v>
@@ -3858,21 +4085,41 @@
     </row>
     <row r="18" spans="1:6" ht="15">
       <c r="A18" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B18" t="s">
-        <v>155</v>
+        <v>143</v>
       </c>
       <c r="C18" t="s">
         <v>24</v>
       </c>
       <c r="D18" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E18" t="s">
-        <v>117</v>
+        <v>162</v>
       </c>
       <c r="F18" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" ht="15">
+      <c r="A19" t="s">
+        <v>122</v>
+      </c>
+      <c r="B19" t="s">
+        <v>163</v>
+      </c>
+      <c r="C19" t="s">
+        <v>24</v>
+      </c>
+      <c r="D19" t="s">
+        <v>152</v>
+      </c>
+      <c r="E19" t="s">
+        <v>116</v>
+      </c>
+      <c r="F19" t="s">
         <v>18</v>
       </c>
     </row>

</xml_diff>